<commit_message>
in progress of adding records
</commit_message>
<xml_diff>
--- a/ML-herb-recognition-DANE.xlsx
+++ b/ML-herb-recognition-DANE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kasia\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kasia\Desktop\ML-herb-recognition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E4DFD3-1C65-4F91-9772-21ABD5A0BE2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548CD3C7-283D-474B-A963-48D69B6D940E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="0" windowWidth="14400" windowHeight="15750" firstSheet="8" activeTab="11" xr2:uid="{54BFF693-94BF-4C22-9B72-2C8DB4535EB5}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="6252" firstSheet="11" activeTab="14" xr2:uid="{54BFF693-94BF-4C22-9B72-2C8DB4535EB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Colors" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,14 @@
     <sheet name="Diseases" sheetId="10" r:id="rId10"/>
     <sheet name="ProductTypes" sheetId="11" r:id="rId11"/>
     <sheet name="Products" sheetId="12" r:id="rId12"/>
+    <sheet name="Poisonability" sheetId="13" r:id="rId13"/>
+    <sheet name="Saps" sheetId="14" r:id="rId14"/>
+    <sheet name="Roots" sheetId="15" r:id="rId15"/>
+    <sheet name="Stalks" sheetId="16" r:id="rId16"/>
+    <sheet name="Hats" sheetId="17" r:id="rId17"/>
+    <sheet name="Fruits" sheetId="19" r:id="rId18"/>
+    <sheet name="Flowers" sheetId="18" r:id="rId19"/>
+    <sheet name="Leafes" sheetId="20" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="231">
   <si>
     <t>Id</t>
   </si>
@@ -621,6 +629,114 @@
   </si>
   <si>
     <t>gastric reflux (in excess)</t>
+  </si>
+  <si>
+    <t>May cause mild irritation or allergic reaction</t>
+  </si>
+  <si>
+    <t>Can cause nausea, vomiting or skin irritation</t>
+  </si>
+  <si>
+    <t>Toxic - causes serious symptoms like dizziness, strong vomiting, diarrhea</t>
+  </si>
+  <si>
+    <t>Highly toxic - can cause organ damage, breathing problems</t>
+  </si>
+  <si>
+    <t>Extremely toxic - can cause paralysis or death</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Occurance</t>
+  </si>
+  <si>
+    <t>ActiveSubstance</t>
+  </si>
+  <si>
+    <t>Symptoms</t>
+  </si>
+  <si>
+    <t>Property</t>
+  </si>
+  <si>
+    <t>ActiveSubstanceId</t>
+  </si>
+  <si>
+    <t>DiseaseId</t>
+  </si>
+  <si>
+    <t>Recipe</t>
+  </si>
+  <si>
+    <t>HealthPrepertyId</t>
+  </si>
+  <si>
+    <t>Contraindication</t>
+  </si>
+  <si>
+    <t>ProductTypeId</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>ColorId</t>
+  </si>
+  <si>
+    <t>LeavesStain</t>
+  </si>
+  <si>
+    <t>Sticky</t>
+  </si>
+  <si>
+    <t>Transparent</t>
+  </si>
+  <si>
+    <t>SurfaceId</t>
+  </si>
+  <si>
+    <t>ThicknessId</t>
+  </si>
+  <si>
+    <t>ShapeId</t>
+  </si>
+  <si>
+    <t>Colord</t>
+  </si>
+  <si>
+    <t>HasSpots</t>
+  </si>
+  <si>
+    <t>HasGills</t>
+  </si>
+  <si>
+    <t>FlavourId</t>
+  </si>
+  <si>
+    <t>SizeInCm</t>
+  </si>
+  <si>
+    <t>ScentPower</t>
+  </si>
+  <si>
+    <t>Stripes</t>
+  </si>
+  <si>
+    <t>Spots</t>
+  </si>
+  <si>
+    <t>Holes</t>
+  </si>
+  <si>
+    <t>LeafShapeId</t>
+  </si>
+  <si>
+    <t>LeafColorId</t>
+  </si>
+  <si>
+    <t>Length</t>
   </si>
 </sst>
 </file>
@@ -1169,8 +1285,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DE7099B-A5EE-4FEF-AF3C-A70CEA02357C}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -1656,6 +1775,23 @@
         <v>0</v>
       </c>
       <c r="F27" s="25"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>215</v>
+      </c>
+      <c r="C28">
+        <v>255</v>
+      </c>
+      <c r="D28">
+        <v>255</v>
+      </c>
+      <c r="E28">
+        <v>255</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1664,7 +1800,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD69ACC-7089-4C80-BCCC-8DD32D0E1BE1}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
@@ -1672,167 +1808,178 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
+      <c r="A1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>200</v>
       </c>
       <c r="C1" t="s">
-        <v>146</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C15" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16">
         <v>15</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>145</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" t="s">
         <v>160</v>
       </c>
     </row>
@@ -1843,86 +1990,94 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67C958BD-C3BB-4904-95E2-B63C538D4002}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
+      <c r="A1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>161</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>170</v>
       </c>
     </row>
@@ -1933,87 +2088,87 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E0106E1-19BC-432B-BBC0-1EE795D91FB1}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
+      <c r="A1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C1" t="s">
-        <v>179</v>
-      </c>
-      <c r="D1">
-        <v>14</v>
+        <v>207</v>
+      </c>
+      <c r="D1" t="s">
+        <v>208</v>
       </c>
       <c r="E1" t="s">
-        <v>180</v>
-      </c>
-      <c r="F1">
-        <v>4</v>
+        <v>209</v>
+      </c>
+      <c r="F1" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D2">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D3">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>182</v>
+      </c>
+      <c r="F3">
         <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>173</v>
-      </c>
-      <c r="C3" t="s">
-        <v>183</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3" t="s">
-        <v>184</v>
-      </c>
-      <c r="F3">
-        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D4">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E4" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F4">
         <v>6</v>
@@ -2021,19 +2176,1183 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D5">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>186</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>5</v>
       </c>
+      <c r="B6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
+        <v>188</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C7" t="s">
+        <v>189</v>
+      </c>
+      <c r="D7">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>190</v>
+      </c>
+      <c r="F7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>177</v>
+      </c>
+      <c r="C8" t="s">
+        <v>191</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>192</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>178</v>
+      </c>
+      <c r="C9" t="s">
+        <v>193</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>194</v>
+      </c>
+      <c r="F9">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCB4CD88-D179-43E7-BB63-6B824B86F15A}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
       <c r="B5" t="s">
-        <v>175</v>
-      </c>
-      <c r="C5" t="s">
-        <v>187</v>
+        <v>198</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>199</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{076C40C8-EF65-4769-AF79-AA7EEC1E1443}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>27</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>20</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEB5C179-228C-4CB2-B374-262D26063ABD}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" t="s">
+        <v>216</v>
+      </c>
+      <c r="D1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>20</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>9</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{367B381E-38AC-4871-B3A2-9E2A1FF070AB}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1" t="s">
+        <v>219</v>
+      </c>
+      <c r="D1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>21</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>20</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>11</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>9</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>21</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E8B1E79-47AC-47D7-AA16-C4544973F7C8}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E1" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" t="s">
+        <v>220</v>
+      </c>
+      <c r="G1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>9</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>9</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>6</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>20</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>8</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>12</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>10</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>4</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>26</v>
+      </c>
+      <c r="C11">
+        <v>9</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>6</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2613C7F2-C6FE-4D63-BAFE-9347DB4EFFBF}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E1" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>21</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>6</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>16</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7">
+        <v>9</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>14</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>12</v>
+      </c>
+      <c r="C10">
+        <v>6</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>8</v>
+      </c>
+      <c r="D11">
+        <v>11</v>
+      </c>
+      <c r="E11">
+        <v>5</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{656FEA14-A5E7-4F2E-8444-7E710722E66F}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D1" t="s">
+        <v>218</v>
+      </c>
+      <c r="E1" t="s">
+        <v>222</v>
+      </c>
+      <c r="F1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>8</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>11</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>11</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>6</v>
+      </c>
+      <c r="C5">
+        <v>5</v>
       </c>
       <c r="D5">
         <v>9</v>
       </c>
-      <c r="E5" t="s">
-        <v>188</v>
+      <c r="E5">
+        <v>13</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -2041,62 +3360,122 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>176</v>
-      </c>
-      <c r="C6" t="s">
-        <v>189</v>
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>12</v>
       </c>
       <c r="D6">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>190</v>
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>16</v>
       </c>
       <c r="F6">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>177</v>
-      </c>
-      <c r="C7" t="s">
-        <v>191</v>
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
       </c>
       <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7" t="s">
-        <v>192</v>
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>9</v>
       </c>
       <c r="F7">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <v>15</v>
+      </c>
+      <c r="D8">
         <v>8</v>
       </c>
-      <c r="B8" t="s">
-        <v>178</v>
-      </c>
-      <c r="C8" t="s">
-        <v>193</v>
-      </c>
-      <c r="D8">
-        <v>7</v>
-      </c>
-      <c r="E8" t="s">
-        <v>194</v>
+      <c r="E8">
+        <v>16</v>
       </c>
       <c r="F8">
-        <v>7</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>14</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>6</v>
+      </c>
+      <c r="C10">
+        <v>6</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>8</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>6</v>
+      </c>
+      <c r="E11">
+        <v>16</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2267,6 +3646,335 @@
       </c>
       <c r="B20" t="s">
         <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DF5D3C7-25A6-4106-B925-CEC58F390415}">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E1" t="s">
+        <v>228</v>
+      </c>
+      <c r="F1" t="s">
+        <v>229</v>
+      </c>
+      <c r="G1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H1" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>21</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3">
+        <v>22</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>10</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>9</v>
+      </c>
+      <c r="F4">
+        <v>21</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>15</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>8</v>
+      </c>
+      <c r="F5">
+        <v>20</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5">
+        <v>20</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6">
+        <v>21</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>12</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>21</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>6</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>21</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8">
+        <v>10</v>
+      </c>
+      <c r="I8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>21</v>
+      </c>
+      <c r="G9">
+        <v>9</v>
+      </c>
+      <c r="H9">
+        <v>25</v>
+      </c>
+      <c r="I9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>20</v>
+      </c>
+      <c r="G10">
+        <v>9</v>
+      </c>
+      <c r="H10">
+        <v>8</v>
+      </c>
+      <c r="I10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>8</v>
+      </c>
+      <c r="F11">
+        <v>20</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>12</v>
+      </c>
+      <c r="I11">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2541,30 +4249,38 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9445F368-8D53-4A3D-8CAF-659CA5173E8A}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
+      <c r="A1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>79</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>80</v>
       </c>
     </row>
@@ -2575,121 +4291,129 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBEE78D5-2CDE-41DE-9483-E092B1F07510}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
+      <c r="A1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>82</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15">
         <v>14</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>95</v>
       </c>
     </row>
@@ -2700,169 +4424,177 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C715A7-525F-48C4-8B06-D2CEA214127A}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
+      <c r="A1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>96</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21">
         <v>20</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>115</v>
       </c>
     </row>
@@ -2873,175 +4605,235 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5036F7A8-2D27-4F40-A907-03AB38823BF9}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>116</v>
       </c>
-      <c r="C1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>117</v>
       </c>
-      <c r="C2">
+      <c r="C3">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
+      <c r="D3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>118</v>
       </c>
-      <c r="C3">
+      <c r="C4">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4">
+      <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>119</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5">
+      <c r="D5">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
         <v>120</v>
       </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6">
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>121</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7">
+      <c r="D7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>122</v>
       </c>
-      <c r="C7">
+      <c r="C8">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8">
+      <c r="D8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>123</v>
       </c>
-      <c r="C8">
+      <c r="C9">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9">
+      <c r="D9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>124</v>
       </c>
-      <c r="C9">
+      <c r="C10">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10">
+      <c r="D10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>125</v>
       </c>
-      <c r="C10">
+      <c r="C11">
         <v>4</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11">
+      <c r="D11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12">
         <v>11</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>126</v>
       </c>
-      <c r="C11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12">
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
         <v>12</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>127</v>
       </c>
-      <c r="C12">
+      <c r="C13">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13">
+      <c r="D13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
         <v>13</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>128</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14">
+      <c r="D14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
         <v>14</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>129</v>
       </c>
-      <c r="C14">
+      <c r="C15">
         <v>5</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15">
+      <c r="D15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16">
         <v>15</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>130</v>
       </c>
-      <c r="C15">
+      <c r="C16">
         <v>16</v>
+      </c>
+      <c r="D16">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mark with colours inserted data
</commit_message>
<xml_diff>
--- a/ML-herb-recognition-DANE.xlsx
+++ b/ML-herb-recognition-DANE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kasia\Desktop\ML-herb-recognition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3C8FA92-4984-40FB-82AE-C8B7B5733F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967790D5-4735-4227-A62F-F133B2EC31C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="930" firstSheet="1" activeTab="1" xr2:uid="{54BFF693-94BF-4C22-9B72-2C8DB4535EB5}"/>
+    <workbookView xWindow="-14400" yWindow="0" windowWidth="14400" windowHeight="15750" tabRatio="930" firstSheet="9" activeTab="10" xr2:uid="{54BFF693-94BF-4C22-9B72-2C8DB4535EB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Colors" sheetId="1" r:id="rId1"/>
@@ -1519,6 +1519,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DE7099B-A5EE-4FEF-AF3C-A70CEA02357C}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2260,6 +2263,9 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEB5C179-228C-4CB2-B374-262D26063ABD}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2510,6 +2516,9 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBEE78D5-2CDE-41DE-9483-E092B1F07510}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2651,6 +2660,9 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E8B1E79-47AC-47D7-AA16-C4544973F7C8}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -2753,6 +2765,9 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DF5D3C7-25A6-4106-B925-CEC58F390415}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3022,6 +3037,9 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{656FEA14-A5E7-4F2E-8444-7E710722E66F}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -3192,6 +3210,9 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2613C7F2-C6FE-4D63-BAFE-9347DB4EFFBF}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3386,6 +3407,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{711C130C-398C-48F7-B440-F4EF1EDFE1A8}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4465,6 +4489,9 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5036F7A8-2D27-4F40-A907-03AB38823BF9}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4780,6 +4807,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D13DE7AB-A127-4693-876C-B5F4C914E2E1}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4873,6 +4903,9 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07D2D1C2-BC6F-49A2-914C-E738466089FA}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -4971,6 +5004,9 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E0D2913-F7D8-4615-A16A-1B5D75758C41}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -5087,6 +5123,9 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C715A7-525F-48C4-8B06-D2CEA214127A}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5268,6 +5307,9 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD69ACC-7089-4C80-BCCC-8DD32D0E1BE1}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
added userInput table to store temporary data given by user
</commit_message>
<xml_diff>
--- a/ML-herb-recognition-DANE.xlsx
+++ b/ML-herb-recognition-DANE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kasia\Desktop\ML-herb-recognition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967790D5-4735-4227-A62F-F133B2EC31C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB5EDE1-D502-4A01-A250-55A394218927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14400" yWindow="0" windowWidth="14400" windowHeight="15750" tabRatio="930" firstSheet="9" activeTab="10" xr2:uid="{54BFF693-94BF-4C22-9B72-2C8DB4535EB5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="930" firstSheet="7" activeTab="22" xr2:uid="{54BFF693-94BF-4C22-9B72-2C8DB4535EB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Colors" sheetId="1" r:id="rId1"/>
@@ -2038,7 +2038,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E0106E1-19BC-432B-BBC0-1EE795D91FB1}">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
+    <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2177,6 +2177,9 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{076C40C8-EF65-4769-AF79-AA7EEC1E1443}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2380,6 +2383,9 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{367B381E-38AC-4871-B3A2-9E2A1FF070AB}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -3346,6 +3352,9 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCB4CD88-D179-43E7-BB63-6B824B86F15A}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3584,7 +3593,7 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52F7ADAA-D38B-4FD0-A7F1-B1E355747A12}">
   <sheetPr>
-    <tabColor rgb="FF32CD32"/>
+    <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="A1:P11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4163,6 +4172,9 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45929B25-8F0F-4486-806B-5E96332ADC13}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5081,6 +5093,9 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9445F368-8D53-4A3D-8CAF-659CA5173E8A}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -5500,6 +5515,9 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67C958BD-C3BB-4904-95E2-B63C538D4002}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>